<commit_message>
file manager tc's and conveyor inspect tc's added
</commit_message>
<xml_diff>
--- a/src/main/resources/excel_data/ConveyorUpload.xlsx
+++ b/src/main/resources/excel_data/ConveyorUpload.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10312"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10211"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65708513-27AB-614E-99CE-A0C98F3705D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A84D5B-B33F-7A44-BEEA-1F41BBED170A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1252,13 +1252,13 @@
     <t>Mechanical</t>
   </si>
   <si>
+    <t>Dual drive 381</t>
+  </si>
+  <si>
+    <t>5,3,3</t>
+  </si>
+  <si>
     <t>601</t>
-  </si>
-  <si>
-    <t>Dual drive 381</t>
-  </si>
-  <si>
-    <t>5,3,3</t>
   </si>
   <si>
     <t>2.6</t>
@@ -1651,6 +1651,7 @@
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="28" max="28" width="11.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -1982,7 +1983,7 @@
         <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D4">
         <v>23</v>
@@ -2003,7 +2004,7 @@
         <v>23</v>
       </c>
       <c r="J4" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="K4">
         <v>24</v>
@@ -2024,7 +2025,7 @@
         <v>144</v>
       </c>
       <c r="Q4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="R4" t="s">
         <v>147</v>

</xml_diff>